<commit_message>
Add rates for Christopher Perez, Johnley Theagene and Ryan Willis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K1L8ax2xDGcRuftFbYF5za
</commit_message>
<xml_diff>
--- a/payroll/2026-10-02/305SKY_Payroll_2026-10-02_to_2026-10-08.xlsx
+++ b/payroll/2026-10-02/305SKY_Payroll_2026-10-02_to_2026-10-08.xlsx
@@ -157,7 +157,7 @@
     <t xml:space="preserve">Mike Markley</t>
   </si>
   <si>
-    <t xml:space="preserve">RATE NOT ON RATE SHEET</t>
+    <t xml:space="preserve">Rate given by Stephanie 2026-10-09</t>
   </si>
   <si>
     <t xml:space="preserve">Location</t>
@@ -372,7 +372,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -474,10 +474,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -824,9 +820,9 @@
       <c r="B8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="8" t="str">
+      <c r="C8" s="8" t="n">
         <f aca="false">IFERROR(IF(INDEX(Rates!$B$2:$B$14,MATCH(A8,Rates!$A$2:$A$14,0))="","",INDEX(Rates!$B$2:$B$14,MATCH(A8,Rates!$A$2:$A$14,0))),"")</f>
-        <v/>
+        <v>36</v>
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">ROUND(SUMIFS('Hours Detail'!$J$2:$J$13,'Hours Detail'!$A$2:$A$13,A8),2)</f>
@@ -848,21 +844,21 @@
         <f aca="false">ROUND(MAX(F8-$B$4,0),2)</f>
         <v>0</v>
       </c>
-      <c r="I8" s="11" t="str">
+      <c r="I8" s="11" t="n">
         <f aca="false">IF(C8="","",ROUND(G8*C8,2))</f>
-        <v/>
-      </c>
-      <c r="J8" s="11" t="str">
+        <v>1238.4</v>
+      </c>
+      <c r="J8" s="11" t="n">
         <f aca="false">IF(C8="","",ROUND(H8*C8*$B$5,2))</f>
-        <v/>
-      </c>
-      <c r="K8" s="12" t="str">
+        <v>0</v>
+      </c>
+      <c r="K8" s="12" t="n">
         <f aca="false">IF(C8="","",I8+J8)</f>
-        <v/>
+        <v>1238.4</v>
       </c>
       <c r="L8" s="13" t="str">
         <f aca="false">IF(C8="","RATE NEEDED",IF(E8&gt;0,"Hours withheld — confirm",""))</f>
-        <v>RATE NEEDED</v>
+        <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -968,9 +964,9 @@
       <c r="B11" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="8" t="str">
+      <c r="C11" s="8" t="n">
         <f aca="false">IFERROR(IF(INDEX(Rates!$B$2:$B$14,MATCH(A11,Rates!$A$2:$A$14,0))="","",INDEX(Rates!$B$2:$B$14,MATCH(A11,Rates!$A$2:$A$14,0))),"")</f>
-        <v/>
+        <v>26</v>
       </c>
       <c r="D11" s="9" t="n">
         <f aca="false">ROUND(SUMIFS('Hours Detail'!$J$2:$J$13,'Hours Detail'!$A$2:$A$13,A11),2)</f>
@@ -992,21 +988,21 @@
         <f aca="false">ROUND(MAX(F11-$B$4,0),2)</f>
         <v>3.4</v>
       </c>
-      <c r="I11" s="11" t="str">
+      <c r="I11" s="11" t="n">
         <f aca="false">IF(C11="","",ROUND(G11*C11,2))</f>
-        <v/>
-      </c>
-      <c r="J11" s="11" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J11" s="11" t="n">
         <f aca="false">IF(C11="","",ROUND(H11*C11*$B$5,2))</f>
-        <v/>
-      </c>
-      <c r="K11" s="12" t="str">
+        <v>132.6</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <f aca="false">IF(C11="","",I11+J11)</f>
-        <v/>
+        <v>1172.6</v>
       </c>
       <c r="L11" s="13" t="str">
         <f aca="false">IF(C11="","RATE NEEDED",IF(E11&gt;0,"Hours withheld — confirm",""))</f>
-        <v>RATE NEEDED</v>
+        <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1304,9 +1300,9 @@
       <c r="B18" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="8" t="str">
+      <c r="C18" s="8" t="n">
         <f aca="false">IFERROR(IF(INDEX(Rates!$B$2:$B$14,MATCH(A18,Rates!$A$2:$A$14,0))="","",INDEX(Rates!$B$2:$B$14,MATCH(A18,Rates!$A$2:$A$14,0))),"")</f>
-        <v/>
+        <v>30</v>
       </c>
       <c r="D18" s="9" t="n">
         <f aca="false">ROUND(SUMIFS('Hours Detail'!$J$2:$J$13,'Hours Detail'!$A$2:$A$13,A18),2)</f>
@@ -1328,21 +1324,21 @@
         <f aca="false">ROUND(MAX(F18-$B$4,0),2)</f>
         <v>6.4</v>
       </c>
-      <c r="I18" s="11" t="str">
+      <c r="I18" s="11" t="n">
         <f aca="false">IF(C18="","",ROUND(G18*C18,2))</f>
-        <v/>
-      </c>
-      <c r="J18" s="11" t="str">
+        <v>1200</v>
+      </c>
+      <c r="J18" s="11" t="n">
         <f aca="false">IF(C18="","",ROUND(H18*C18*$B$5,2))</f>
-        <v/>
-      </c>
-      <c r="K18" s="12" t="str">
+        <v>288</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <f aca="false">IF(C18="","",I18+J18)</f>
-        <v/>
+        <v>1488</v>
       </c>
       <c r="L18" s="13" t="str">
         <f aca="false">IF(C18="","RATE NEEDED",IF(E18&gt;0,"Hours withheld — confirm",""))</f>
-        <v>RATE NEEDED</v>
+        <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1373,19 +1369,19 @@
       </c>
       <c r="I19" s="17" t="n">
         <f aca="false">SUM(I8:I18)</f>
-        <v>8532.6</v>
+        <v>12011</v>
       </c>
       <c r="J19" s="17" t="n">
         <f aca="false">SUM(J8:J18)</f>
-        <v>1174.5</v>
+        <v>1595.1</v>
       </c>
       <c r="K19" s="17" t="n">
         <f aca="false">SUM(K8:K18)</f>
-        <v>9707.1</v>
+        <v>13606.1</v>
       </c>
       <c r="L19" s="18" t="str">
         <f aca="false">IF(COUNTIF(L8:L18,"RATE NEEDED")&gt;0,COUNTIF(L8:L18,"RATE NEEDED")&amp;" rate(s) missing — total incomplete","")</f>
-        <v>3 rate(s) missing — total incomplete</v>
+        <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1472,13 +1468,13 @@
         <f aca="false">SUMIFS(Payroll!$H$8:$H$18,Payroll!$A$8:$A$18,A4)</f>
         <v>0</v>
       </c>
-      <c r="D4" s="21" t="str">
+      <c r="D4" s="21" t="n">
         <f aca="false">INDEX(Payroll!$C$8:$C$18,MATCH(A4,Payroll!$A$8:$A$18,0))</f>
-        <v/>
-      </c>
-      <c r="E4" s="22" t="str">
+        <v>36</v>
+      </c>
+      <c r="E4" s="22" t="n">
         <f aca="false">IF(D4="","RATE NEEDED",SUMIFS(Payroll!$K$8:$K$18,Payroll!$A$8:$A$18,A4))</f>
-        <v>RATE NEEDED</v>
+        <v>1238.4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1535,13 +1531,13 @@
         <f aca="false">SUMIFS(Payroll!$H$8:$H$18,Payroll!$A$8:$A$18,A7)</f>
         <v>3.4</v>
       </c>
-      <c r="D7" s="21" t="str">
+      <c r="D7" s="21" t="n">
         <f aca="false">INDEX(Payroll!$C$8:$C$18,MATCH(A7,Payroll!$A$8:$A$18,0))</f>
-        <v/>
-      </c>
-      <c r="E7" s="22" t="str">
+        <v>26</v>
+      </c>
+      <c r="E7" s="22" t="n">
         <f aca="false">IF(D7="","RATE NEEDED",SUMIFS(Payroll!$K$8:$K$18,Payroll!$A$8:$A$18,A7))</f>
-        <v>RATE NEEDED</v>
+        <v>1172.6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1682,13 +1678,13 @@
         <f aca="false">SUMIFS(Payroll!$H$8:$H$18,Payroll!$A$8:$A$18,A14)</f>
         <v>6.4</v>
       </c>
-      <c r="D14" s="21" t="str">
+      <c r="D14" s="21" t="n">
         <f aca="false">INDEX(Payroll!$C$8:$C$18,MATCH(A14,Payroll!$A$8:$A$18,0))</f>
-        <v/>
-      </c>
-      <c r="E14" s="22" t="str">
+        <v>30</v>
+      </c>
+      <c r="E14" s="22" t="n">
         <f aca="false">IF(D14="","RATE NEEDED",SUMIFS(Payroll!$K$8:$K$18,Payroll!$A$8:$A$18,A14))</f>
-        <v>RATE NEEDED</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1706,7 +1702,7 @@
       <c r="D15" s="15"/>
       <c r="E15" s="17" t="n">
         <f aca="false">SUM(E4:E14)</f>
-        <v>9707.1</v>
+        <v>13606.1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1881,7 +1877,9 @@
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="26"/>
+      <c r="B12" s="23" t="n">
+        <v>36</v>
+      </c>
       <c r="C12" s="24" t="n">
         <v>0</v>
       </c>
@@ -1893,7 +1891,9 @@
       <c r="A13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="26"/>
+      <c r="B13" s="23" t="n">
+        <v>26</v>
+      </c>
       <c r="C13" s="24" t="n">
         <v>0</v>
       </c>
@@ -1905,7 +1905,9 @@
       <c r="A14" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="26"/>
+      <c r="B14" s="23" t="n">
+        <v>30</v>
+      </c>
       <c r="C14" s="24" t="n">
         <v>0</v>
       </c>
@@ -1998,7 +2000,7 @@
       <c r="I2" s="24" t="n">
         <v>11.3</v>
       </c>
-      <c r="J2" s="27" t="n">
+      <c r="J2" s="26" t="n">
         <f aca="false">SUM(C2:I2)</f>
         <v>34.4</v>
       </c>
@@ -2032,7 +2034,7 @@
       <c r="I3" s="24" t="n">
         <v>8.3</v>
       </c>
-      <c r="J3" s="27" t="n">
+      <c r="J3" s="26" t="n">
         <f aca="false">SUM(C3:I3)</f>
         <v>41.5</v>
       </c>
@@ -2066,7 +2068,7 @@
       <c r="I4" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="J4" s="27" t="n">
+      <c r="J4" s="26" t="n">
         <f aca="false">SUM(C4:I4)</f>
         <v>39.8</v>
       </c>
@@ -2100,7 +2102,7 @@
       <c r="I5" s="24" t="n">
         <v>11.2</v>
       </c>
-      <c r="J5" s="27" t="n">
+      <c r="J5" s="26" t="n">
         <f aca="false">SUM(C5:I5)</f>
         <v>34.8</v>
       </c>
@@ -2128,7 +2130,7 @@
       <c r="G6" s="24"/>
       <c r="H6" s="24"/>
       <c r="I6" s="24"/>
-      <c r="J6" s="27" t="n">
+      <c r="J6" s="26" t="n">
         <f aca="false">SUM(C6:I6)</f>
         <v>8.6</v>
       </c>
@@ -2162,7 +2164,7 @@
       <c r="I7" s="24" t="n">
         <v>9.7</v>
       </c>
-      <c r="J7" s="27" t="n">
+      <c r="J7" s="26" t="n">
         <f aca="false">SUM(C7:I7)</f>
         <v>45.7</v>
       </c>
@@ -2198,7 +2200,7 @@
       <c r="I8" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="J8" s="27" t="n">
+      <c r="J8" s="26" t="n">
         <f aca="false">SUM(C8:I8)</f>
         <v>36.6</v>
       </c>
@@ -2228,7 +2230,7 @@
         <v>7.9</v>
       </c>
       <c r="I9" s="24"/>
-      <c r="J9" s="27" t="n">
+      <c r="J9" s="26" t="n">
         <f aca="false">SUM(C9:I9)</f>
         <v>23.4</v>
       </c>
@@ -2264,7 +2266,7 @@
       <c r="I10" s="24" t="n">
         <v>7.9</v>
       </c>
-      <c r="J10" s="27" t="n">
+      <c r="J10" s="26" t="n">
         <f aca="false">SUM(C10:I10)</f>
         <v>44.1</v>
       </c>
@@ -2300,7 +2302,7 @@
       <c r="I11" s="24" t="n">
         <v>7.8</v>
       </c>
-      <c r="J11" s="27" t="n">
+      <c r="J11" s="26" t="n">
         <f aca="false">SUM(C11:I11)</f>
         <v>44.4</v>
       </c>
@@ -2336,7 +2338,7 @@
       <c r="I12" s="24" t="n">
         <v>9.9</v>
       </c>
-      <c r="J12" s="27" t="n">
+      <c r="J12" s="26" t="n">
         <f aca="false">SUM(C12:I12)</f>
         <v>50.4</v>
       </c>
@@ -2370,7 +2372,7 @@
       <c r="I13" s="24" t="n">
         <v>9.3</v>
       </c>
-      <c r="J13" s="27" t="n">
+      <c r="J13" s="26" t="n">
         <f aca="false">SUM(C13:I13)</f>
         <v>46.4</v>
       </c>

</xml_diff>

<commit_message>
Stop withholding 10 hours from Mateo Moreno
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K1L8ax2xDGcRuftFbYF5za
</commit_message>
<xml_diff>
--- a/payroll/2026-10-02/305SKY_Payroll_2026-10-02_to_2026-10-08.xlsx
+++ b/payroll/2026-10-02/305SKY_Payroll_2026-10-02_to_2026-10-08.xlsx
@@ -151,7 +151,7 @@
     <t xml:space="preserve">Tom Marshal</t>
   </si>
   <si>
-    <t xml:space="preserve">Rate sheet note: "withold 10 Hours" (confirm whether one-time or every period)</t>
+    <t xml:space="preserve">Rate sheet says "withold 10 Hours" — not applied (per Stephanie 2026-10-09)</t>
   </si>
   <si>
     <t xml:space="preserve">Mike Markley</t>
@@ -372,7 +372,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -470,10 +470,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1118,15 +1114,15 @@
       </c>
       <c r="E14" s="9" t="n">
         <f aca="false">IFERROR(INDEX(Rates!$C$2:$C$14,MATCH(A14,Rates!$A$2:$A$14,0)),0)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F14" s="10" t="n">
         <f aca="false">ROUND(MAX(D14-E14,0),2)</f>
-        <v>13.4</v>
+        <v>23.4</v>
       </c>
       <c r="G14" s="10" t="n">
         <f aca="false">MIN(F14,$B$4)</f>
-        <v>13.4</v>
+        <v>23.4</v>
       </c>
       <c r="H14" s="10" t="n">
         <f aca="false">ROUND(MAX(F14-$B$4,0),2)</f>
@@ -1134,7 +1130,7 @@
       </c>
       <c r="I14" s="11" t="n">
         <f aca="false">IF(C14="","",ROUND(G14*C14,2))</f>
-        <v>268</v>
+        <v>468</v>
       </c>
       <c r="J14" s="11" t="n">
         <f aca="false">IF(C14="","",ROUND(H14*C14*$B$5,2))</f>
@@ -1142,11 +1138,11 @@
       </c>
       <c r="K14" s="12" t="n">
         <f aca="false">IF(C14="","",I14+J14)</f>
-        <v>268</v>
+        <v>468</v>
       </c>
       <c r="L14" s="13" t="str">
         <f aca="false">IF(C14="","RATE NEEDED",IF(E14&gt;0,"Hours withheld — confirm",""))</f>
-        <v>Hours withheld — confirm</v>
+        <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1353,15 +1349,15 @@
       </c>
       <c r="E19" s="16" t="n">
         <f aca="false">SUM(E8:E18)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F19" s="16" t="n">
         <f aca="false">SUM(F8:F18)</f>
-        <v>440.1</v>
+        <v>450.1</v>
       </c>
       <c r="G19" s="16" t="n">
         <f aca="false">SUM(G8:G18)</f>
-        <v>404.2</v>
+        <v>414.2</v>
       </c>
       <c r="H19" s="16" t="n">
         <f aca="false">SUM(H8:H18)</f>
@@ -1369,7 +1365,7 @@
       </c>
       <c r="I19" s="17" t="n">
         <f aca="false">SUM(I8:I18)</f>
-        <v>12011</v>
+        <v>12211</v>
       </c>
       <c r="J19" s="17" t="n">
         <f aca="false">SUM(J8:J18)</f>
@@ -1377,7 +1373,7 @@
       </c>
       <c r="K19" s="17" t="n">
         <f aca="false">SUM(K8:K18)</f>
-        <v>13606.1</v>
+        <v>13806.1</v>
       </c>
       <c r="L19" s="18" t="str">
         <f aca="false">IF(COUNTIF(L8:L18,"RATE NEEDED")&gt;0,COUNTIF(L8:L18,"RATE NEEDED")&amp;" rate(s) missing — total incomplete","")</f>
@@ -1588,7 +1584,7 @@
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">SUMIFS(Payroll!$G$8:$G$18,Payroll!$A$8:$A$18,A10)</f>
-        <v>13.4</v>
+        <v>23.4</v>
       </c>
       <c r="C10" s="20" t="n">
         <f aca="false">SUMIFS(Payroll!$H$8:$H$18,Payroll!$A$8:$A$18,A10)</f>
@@ -1600,7 +1596,7 @@
       </c>
       <c r="E10" s="22" t="n">
         <f aca="false">IF(D10="","RATE NEEDED",SUMIFS(Payroll!$K$8:$K$18,Payroll!$A$8:$A$18,A10))</f>
-        <v>268</v>
+        <v>468</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1693,7 +1689,7 @@
       </c>
       <c r="B15" s="16" t="n">
         <f aca="false">SUM(B4:B14)</f>
-        <v>404.2</v>
+        <v>414.2</v>
       </c>
       <c r="C15" s="16" t="n">
         <f aca="false">SUM(C4:C14)</f>
@@ -1702,7 +1698,7 @@
       <c r="D15" s="15"/>
       <c r="E15" s="17" t="n">
         <f aca="false">SUM(E4:E14)</f>
-        <v>13606.1</v>
+        <v>13806.1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1830,8 +1826,8 @@
       <c r="B8" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="C8" s="25" t="n">
-        <v>10</v>
+      <c r="C8" s="24" t="n">
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>42</v>
@@ -2000,7 +1996,7 @@
       <c r="I2" s="24" t="n">
         <v>11.3</v>
       </c>
-      <c r="J2" s="26" t="n">
+      <c r="J2" s="25" t="n">
         <f aca="false">SUM(C2:I2)</f>
         <v>34.4</v>
       </c>
@@ -2034,7 +2030,7 @@
       <c r="I3" s="24" t="n">
         <v>8.3</v>
       </c>
-      <c r="J3" s="26" t="n">
+      <c r="J3" s="25" t="n">
         <f aca="false">SUM(C3:I3)</f>
         <v>41.5</v>
       </c>
@@ -2068,7 +2064,7 @@
       <c r="I4" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="J4" s="26" t="n">
+      <c r="J4" s="25" t="n">
         <f aca="false">SUM(C4:I4)</f>
         <v>39.8</v>
       </c>
@@ -2102,7 +2098,7 @@
       <c r="I5" s="24" t="n">
         <v>11.2</v>
       </c>
-      <c r="J5" s="26" t="n">
+      <c r="J5" s="25" t="n">
         <f aca="false">SUM(C5:I5)</f>
         <v>34.8</v>
       </c>
@@ -2130,7 +2126,7 @@
       <c r="G6" s="24"/>
       <c r="H6" s="24"/>
       <c r="I6" s="24"/>
-      <c r="J6" s="26" t="n">
+      <c r="J6" s="25" t="n">
         <f aca="false">SUM(C6:I6)</f>
         <v>8.6</v>
       </c>
@@ -2164,7 +2160,7 @@
       <c r="I7" s="24" t="n">
         <v>9.7</v>
       </c>
-      <c r="J7" s="26" t="n">
+      <c r="J7" s="25" t="n">
         <f aca="false">SUM(C7:I7)</f>
         <v>45.7</v>
       </c>
@@ -2200,7 +2196,7 @@
       <c r="I8" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="J8" s="26" t="n">
+      <c r="J8" s="25" t="n">
         <f aca="false">SUM(C8:I8)</f>
         <v>36.6</v>
       </c>
@@ -2230,7 +2226,7 @@
         <v>7.9</v>
       </c>
       <c r="I9" s="24"/>
-      <c r="J9" s="26" t="n">
+      <c r="J9" s="25" t="n">
         <f aca="false">SUM(C9:I9)</f>
         <v>23.4</v>
       </c>
@@ -2266,7 +2262,7 @@
       <c r="I10" s="24" t="n">
         <v>7.9</v>
       </c>
-      <c r="J10" s="26" t="n">
+      <c r="J10" s="25" t="n">
         <f aca="false">SUM(C10:I10)</f>
         <v>44.1</v>
       </c>
@@ -2302,7 +2298,7 @@
       <c r="I11" s="24" t="n">
         <v>7.8</v>
       </c>
-      <c r="J11" s="26" t="n">
+      <c r="J11" s="25" t="n">
         <f aca="false">SUM(C11:I11)</f>
         <v>44.4</v>
       </c>
@@ -2338,7 +2334,7 @@
       <c r="I12" s="24" t="n">
         <v>9.9</v>
       </c>
-      <c r="J12" s="26" t="n">
+      <c r="J12" s="25" t="n">
         <f aca="false">SUM(C12:I12)</f>
         <v>50.4</v>
       </c>
@@ -2372,7 +2368,7 @@
       <c r="I13" s="24" t="n">
         <v>9.3</v>
       </c>
-      <c r="J13" s="26" t="n">
+      <c r="J13" s="25" t="n">
         <f aca="false">SUM(C13:I13)</f>
         <v>46.4</v>
       </c>

</xml_diff>